<commit_message>
2025.01.13_1 Backup from yesterday
</commit_message>
<xml_diff>
--- a/Analysis/Baseline_data_d1_exclusive.xlsx
+++ b/Analysis/Baseline_data_d1_exclusive.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gustavosplmoura/Library/Mobile Documents/com~apple~CloudDocs/Medicina/Biblioteca/Research/Data Science/Data Science/PROJECTS/DVEP/Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A024D2D-567F-554E-BF14-2D0F6DA5FB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D1145D-AA3D-A34A-9F67-4AF1B8F00B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20140" activeTab="2" xr2:uid="{704BFAC6-42D9-C841-B8C7-75AA64A2EC45}"/>
+    <workbookView xWindow="8320" yWindow="500" windowWidth="34560" windowHeight="20140" activeTab="2" xr2:uid="{704BFAC6-42D9-C841-B8C7-75AA64A2EC45}"/>
   </bookViews>
   <sheets>
     <sheet name="data_d1_exclusive" sheetId="2" r:id="rId1"/>
@@ -5770,7 +5770,7 @@
     <col min="3" max="3" width="6.59765625" style="1" customWidth="1"/>
     <col min="4" max="4" width="9.3984375" style="1" customWidth="1"/>
     <col min="5" max="5" width="5.796875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11" style="1"/>
+    <col min="6" max="6" width="8.796875" style="1" customWidth="1"/>
     <col min="7" max="7" width="9.3984375" style="2" customWidth="1"/>
     <col min="8" max="8" width="8.19921875" style="2" customWidth="1"/>
     <col min="9" max="9" width="8" style="2" customWidth="1"/>
@@ -6750,7 +6750,7 @@
     <mergeCell ref="E1:F1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="H2:I51 H53:I1048576 G52:H52">
+  <conditionalFormatting sqref="H2:I51 G52:H52 H53:I1048576">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0.05</formula>
     </cfRule>

</xml_diff>